<commit_message>
removed shank length from .xlsx file
</commit_message>
<xml_diff>
--- a/probe_contours.xlsx
+++ b/probe_contours.xlsx
@@ -595,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -609,11 +609,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -622,9 +617,6 @@
       <c r="B2" t="n">
         <v>6000</v>
       </c>
-      <c r="C2" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -633,9 +625,6 @@
       <c r="B3" t="n">
         <v>257.5</v>
       </c>
-      <c r="C3" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -644,9 +633,6 @@
       <c r="B4" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C4" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -655,9 +641,6 @@
       <c r="B5" t="n">
         <v>-77.5</v>
       </c>
-      <c r="C5" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -666,9 +649,6 @@
       <c r="B6" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C6" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -677,9 +657,6 @@
       <c r="B7" t="n">
         <v>257.5</v>
       </c>
-      <c r="C7" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -687,9 +664,6 @@
       </c>
       <c r="B8" t="n">
         <v>6000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2281,7 +2255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2295,11 +2269,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2308,9 +2277,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2319,9 +2285,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2330,9 +2293,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -2341,9 +2301,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2352,9 +2309,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2363,9 +2317,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2373,9 +2324,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -2389,7 +2337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2403,11 +2351,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2416,9 +2359,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2427,9 +2367,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2438,9 +2375,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -2449,9 +2383,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2460,9 +2391,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2471,9 +2399,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2481,9 +2406,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -6006,7 +5928,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>-14.5</v>
+        <v>-16</v>
       </c>
       <c r="B40" t="n">
         <v>600</v>
@@ -6014,7 +5936,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>-13</v>
+        <v>-16</v>
       </c>
       <c r="B41" t="n">
         <v>400</v>
@@ -6022,7 +5944,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>-11.5</v>
+        <v>-16</v>
       </c>
       <c r="B42" t="n">
         <v>200</v>
@@ -6030,7 +5952,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>-10</v>
+        <v>-16</v>
       </c>
       <c r="B43" t="n">
         <v>0</v>
@@ -6062,7 +5984,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B47" t="n">
         <v>0</v>
@@ -6070,7 +5992,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>11.5</v>
+        <v>16</v>
       </c>
       <c r="B48" t="n">
         <v>200</v>
@@ -6078,7 +6000,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B49" t="n">
         <v>400</v>
@@ -6086,7 +6008,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>14.5</v>
+        <v>16</v>
       </c>
       <c r="B50" t="n">
         <v>600</v>
@@ -11771,7 +11693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11785,11 +11707,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -11798,9 +11715,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -11809,9 +11723,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -11820,9 +11731,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -11831,9 +11739,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -11842,9 +11747,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -11853,9 +11755,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -11863,9 +11762,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -11879,7 +11775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11893,11 +11789,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -11906,9 +11797,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -11917,9 +11805,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -11928,9 +11813,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -11939,9 +11821,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -11950,9 +11829,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -11961,9 +11837,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -11971,9 +11844,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -11987,7 +11857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12001,11 +11871,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -12014,9 +11879,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -12025,9 +11887,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -12036,9 +11895,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -12047,9 +11903,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -12058,9 +11911,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -12069,9 +11919,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -12079,9 +11926,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -12095,7 +11939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12109,11 +11953,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -12122,9 +11961,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -12133,9 +11969,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -12144,9 +11977,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -12155,9 +11985,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -12166,9 +11993,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -12177,9 +12001,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -12187,9 +12008,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -12607,7 +12425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12621,11 +12439,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -12634,9 +12447,6 @@
       <c r="B2" t="n">
         <v>6000</v>
       </c>
-      <c r="C2" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -12645,9 +12455,6 @@
       <c r="B3" t="n">
         <v>257.5</v>
       </c>
-      <c r="C3" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -12656,9 +12463,6 @@
       <c r="B4" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C4" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -12667,9 +12471,6 @@
       <c r="B5" t="n">
         <v>-77.5</v>
       </c>
-      <c r="C5" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -12678,9 +12479,6 @@
       <c r="B6" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C6" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -12689,9 +12487,6 @@
       <c r="B7" t="n">
         <v>257.5</v>
       </c>
-      <c r="C7" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -12699,9 +12494,6 @@
       </c>
       <c r="B8" t="n">
         <v>6000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -12715,7 +12507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12729,11 +12521,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -12742,9 +12529,6 @@
       <c r="B2" t="n">
         <v>9000</v>
       </c>
-      <c r="C2" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -12753,9 +12537,6 @@
       <c r="B3" t="n">
         <v>257.5</v>
       </c>
-      <c r="C3" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -12764,9 +12545,6 @@
       <c r="B4" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C4" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -12775,9 +12553,6 @@
       <c r="B5" t="n">
         <v>-77.5</v>
       </c>
-      <c r="C5" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -12786,9 +12561,6 @@
       <c r="B6" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C6" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -12797,9 +12569,6 @@
       <c r="B7" t="n">
         <v>257.5</v>
       </c>
-      <c r="C7" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -12807,9 +12576,6 @@
       </c>
       <c r="B8" t="n">
         <v>9000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -13883,7 +13649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13897,11 +13663,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -13910,9 +13671,6 @@
       <c r="B2" t="n">
         <v>9000</v>
       </c>
-      <c r="C2" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -13921,9 +13679,6 @@
       <c r="B3" t="n">
         <v>257.5</v>
       </c>
-      <c r="C3" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -13932,9 +13687,6 @@
       <c r="B4" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C4" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -13943,9 +13695,6 @@
       <c r="B5" t="n">
         <v>-77.5</v>
       </c>
-      <c r="C5" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -13954,9 +13703,6 @@
       <c r="B6" t="n">
         <v>-7.5</v>
       </c>
-      <c r="C6" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -13965,9 +13711,6 @@
       <c r="B7" t="n">
         <v>257.5</v>
       </c>
-      <c r="C7" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -13975,9 +13718,6 @@
       </c>
       <c r="B8" t="n">
         <v>9000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -15053,7 +14793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15067,11 +14807,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -15080,9 +14815,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -15091,9 +14823,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -15102,9 +14831,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -15113,9 +14839,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -15124,9 +14847,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -15135,9 +14855,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -15145,9 +14862,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -15161,7 +14875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15175,11 +14889,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -15188,9 +14897,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -15199,9 +14905,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -15210,9 +14913,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -15221,9 +14921,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -15232,9 +14929,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -15243,9 +14937,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -15253,9 +14944,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -15269,7 +14957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15283,11 +14971,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -15296,9 +14979,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -15307,9 +14987,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -15318,9 +14995,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -15329,9 +15003,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -15340,9 +15011,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -15351,9 +15019,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -15361,9 +15026,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -15377,7 +15039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15391,11 +15053,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -15404,9 +15061,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -15415,9 +15069,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -15426,9 +15077,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -15437,9 +15085,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -15448,9 +15093,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -15459,9 +15101,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -15469,9 +15108,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -17691,7 +17327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17705,11 +17341,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -17718,9 +17349,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -17729,9 +17357,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -17740,9 +17365,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -17751,9 +17373,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -17762,9 +17381,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -17773,9 +17389,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -17783,9 +17396,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -17799,7 +17409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17813,11 +17423,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -17826,9 +17431,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -17837,9 +17439,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -17848,9 +17447,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -17859,9 +17455,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -17870,9 +17463,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -17881,9 +17471,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -17891,9 +17478,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -18069,7 +17653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18083,11 +17667,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -18096,9 +17675,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -18107,9 +17683,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -18118,9 +17691,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -18129,9 +17699,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -18140,9 +17707,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -18151,9 +17715,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -18161,9 +17722,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -18177,7 +17735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18191,11 +17749,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -18204,9 +17757,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -18215,9 +17765,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -18226,9 +17773,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -18237,9 +17781,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -18248,9 +17789,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -18259,9 +17797,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -18269,9 +17804,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -21799,7 +21331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21813,11 +21345,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -21826,9 +21353,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -21837,9 +21361,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -21848,9 +21369,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -21859,9 +21377,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -21870,9 +21385,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -21881,9 +21393,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -21891,9 +21400,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -21907,7 +21413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21921,11 +21427,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -21934,9 +21435,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -21945,9 +21443,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -21956,9 +21451,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -21967,9 +21459,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -21978,9 +21467,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -21989,9 +21475,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -21999,9 +21482,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -22015,7 +21495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22029,11 +21509,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -22042,9 +21517,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -22053,9 +21525,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -22064,9 +21533,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -22075,9 +21541,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -22086,9 +21549,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -22097,9 +21557,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -22107,9 +21564,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -22123,7 +21577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22137,11 +21591,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -22150,9 +21599,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -22161,9 +21607,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -22172,9 +21615,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -22183,9 +21623,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -22194,9 +21631,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -22205,9 +21639,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -22215,9 +21646,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -24503,7 +23931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24517,11 +23945,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -24530,9 +23953,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -24541,9 +23961,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -24552,9 +23969,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -24563,9 +23977,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -24574,9 +23985,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -24585,9 +23993,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -24595,9 +24000,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -24611,7 +24013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24625,11 +24027,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -24638,9 +24035,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -24649,9 +24043,6 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -24660,9 +24051,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -24671,9 +24059,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -24682,9 +24067,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -24693,9 +24075,6 @@
       <c r="B7" t="n">
         <v>34</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -24703,9 +24082,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -24719,7 +24095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24733,11 +24109,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -24746,9 +24117,6 @@
       <c r="B2" t="n">
         <v>15000</v>
       </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -24757,9 +24125,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -24768,9 +24133,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -24779,9 +24141,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -24790,9 +24149,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -24801,9 +24157,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -24811,9 +24164,6 @@
       </c>
       <c r="B8" t="n">
         <v>15000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -24827,7 +24177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24841,11 +24191,6 @@
           <t>y</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>shank_length_mm</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -24854,9 +24199,6 @@
       <c r="B2" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -24865,9 +24207,6 @@
       <c r="B3" t="n">
         <v>118</v>
       </c>
-      <c r="C3" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -24876,9 +24215,6 @@
       <c r="B4" t="n">
         <v>-11</v>
       </c>
-      <c r="C4" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -24887,9 +24223,6 @@
       <c r="B5" t="n">
         <v>-156</v>
       </c>
-      <c r="C5" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -24898,9 +24231,6 @@
       <c r="B6" t="n">
         <v>-11</v>
       </c>
-      <c r="C6" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -24909,9 +24239,6 @@
       <c r="B7" t="n">
         <v>118</v>
       </c>
-      <c r="C7" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -24919,9 +24246,6 @@
       </c>
       <c r="B8" t="n">
         <v>30000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>